<commit_message>
Resync phase 7 student profiles from updated Excel.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/student/evening-students/7_phase/eveving cs enginering and medical_governmner.xlsx
+++ b/public/student/evening-students/7_phase/eveving cs enginering and medical_governmner.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\gcp website\final-gcp-website\gcp\Govenment-college-peshawar\public\student\evening-students\7_phase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68CFB458-C063-4FC8-88C3-94906204E4CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FB4E5B4-B7EB-443C-BBF7-2E453E62FE23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="222">
-  <si>
-    <t>Enrollment ID</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="196">
   <si>
     <t>Roll No</t>
   </si>
@@ -61,9 +58,6 @@
     <t>Photo File Name</t>
   </si>
   <si>
-    <t>ENR-202601</t>
-  </si>
-  <si>
     <t>778</t>
   </si>
   <si>
@@ -97,9 +91,6 @@
     <t>778.png</t>
   </si>
   <si>
-    <t>ENR-202602</t>
-  </si>
-  <si>
     <t>775</t>
   </si>
   <si>
@@ -124,9 +115,6 @@
     <t>775.png</t>
   </si>
   <si>
-    <t>ENR-202603</t>
-  </si>
-  <si>
     <t>2162 (Evening)</t>
   </si>
   <si>
@@ -151,9 +139,6 @@
     <t>2162.png</t>
   </si>
   <si>
-    <t>ENR-202604</t>
-  </si>
-  <si>
     <t>2249 (Evening)</t>
   </si>
   <si>
@@ -175,9 +160,6 @@
     <t>2249.png</t>
   </si>
   <si>
-    <t>ENR-202605</t>
-  </si>
-  <si>
     <t>1664</t>
   </si>
   <si>
@@ -202,9 +184,6 @@
     <t>1664.png</t>
   </si>
   <si>
-    <t>ENR-202606</t>
-  </si>
-  <si>
     <t>1668</t>
   </si>
   <si>
@@ -226,9 +205,6 @@
     <t>1668.png</t>
   </si>
   <si>
-    <t>ENR-202607</t>
-  </si>
-  <si>
     <t>M. Yas Barki Zai</t>
   </si>
   <si>
@@ -247,12 +223,6 @@
     <t>Faizullah Town, Gulbarg #4, Peshawar</t>
   </si>
   <si>
-    <t>1671.png</t>
-  </si>
-  <si>
-    <t>ENR-202608</t>
-  </si>
-  <si>
     <t>1679</t>
   </si>
   <si>
@@ -277,9 +247,6 @@
     <t>1679.png</t>
   </si>
   <si>
-    <t>ENR-202609</t>
-  </si>
-  <si>
     <t>1676 (Evening)</t>
   </si>
   <si>
@@ -304,9 +271,6 @@
     <t>1676.png</t>
   </si>
   <si>
-    <t>ENR-202610</t>
-  </si>
-  <si>
     <t>Touseef Ullah</t>
   </si>
   <si>
@@ -325,9 +289,6 @@
     <t>Haryana Bala Shelam, P/Saiban</t>
   </si>
   <si>
-    <t>ENR-202611</t>
-  </si>
-  <si>
     <t>1682</t>
   </si>
   <si>
@@ -352,9 +313,6 @@
     <t>1682.png</t>
   </si>
   <si>
-    <t>ENR-202612</t>
-  </si>
-  <si>
     <t>1663</t>
   </si>
   <si>
@@ -376,9 +334,6 @@
     <t>1663.png</t>
   </si>
   <si>
-    <t>ENR-202613</t>
-  </si>
-  <si>
     <t>1665</t>
   </si>
   <si>
@@ -400,9 +355,6 @@
     <t>1665.png</t>
   </si>
   <si>
-    <t>ENR-202614</t>
-  </si>
-  <si>
     <t>1670</t>
   </si>
   <si>
@@ -424,9 +376,6 @@
     <t>1670.png</t>
   </si>
   <si>
-    <t>ENR-202615</t>
-  </si>
-  <si>
     <t>1673</t>
   </si>
   <si>
@@ -448,9 +397,6 @@
     <t>1673.png</t>
   </si>
   <si>
-    <t>ENR-202616</t>
-  </si>
-  <si>
     <t>1675</t>
   </si>
   <si>
@@ -472,9 +418,6 @@
     <t>1675.png</t>
   </si>
   <si>
-    <t>ENR-202617</t>
-  </si>
-  <si>
     <t>1678 (Evening)</t>
   </si>
   <si>
@@ -496,9 +439,6 @@
     <t>1678.png</t>
   </si>
   <si>
-    <t>ENR-202618</t>
-  </si>
-  <si>
     <t>1681</t>
   </si>
   <si>
@@ -520,9 +460,6 @@
     <t>1681.png</t>
   </si>
   <si>
-    <t>ENR-202619</t>
-  </si>
-  <si>
     <t>1662</t>
   </si>
   <si>
@@ -544,9 +481,6 @@
     <t>1662.png</t>
   </si>
   <si>
-    <t>ENR-202620</t>
-  </si>
-  <si>
     <t>1666</t>
   </si>
   <si>
@@ -568,9 +502,6 @@
     <t>1666.png</t>
   </si>
   <si>
-    <t>ENR-202621</t>
-  </si>
-  <si>
     <t>1669</t>
   </si>
   <si>
@@ -592,9 +523,6 @@
     <t>1669.png</t>
   </si>
   <si>
-    <t>ENR-202622</t>
-  </si>
-  <si>
     <t>1672</t>
   </si>
   <si>
@@ -616,9 +544,6 @@
     <t>1672.png</t>
   </si>
   <si>
-    <t>ENR-202623</t>
-  </si>
-  <si>
     <t>1667</t>
   </si>
   <si>
@@ -640,9 +565,6 @@
     <t>1667.png</t>
   </si>
   <si>
-    <t>ENR-202624</t>
-  </si>
-  <si>
     <t>1677 (Evening)</t>
   </si>
   <si>
@@ -664,9 +586,6 @@
     <t>1677.png</t>
   </si>
   <si>
-    <t>ENR-202625</t>
-  </si>
-  <si>
     <t>1680</t>
   </si>
   <si>
@@ -686,6 +605,9 @@
   </si>
   <si>
     <t>1680.png</t>
+  </si>
+  <si>
+    <t>1674.png</t>
   </si>
 </sst>
 </file>
@@ -1077,10 +999,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="1" max="1" width="19" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="4" width="21" customWidth="1"/>
@@ -1092,1025 +1014,946 @@
     <col min="10" max="10" width="27" customWidth="1"/>
     <col min="11" max="11" width="63" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="J2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="L2" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="E3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>29</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="I3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="J3" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="K3" s="4" t="s">
+      <c r="C4" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="L3" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M3" s="4" t="s">
+      <c r="D4" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="E4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="J4" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="K4" s="2" t="s">
+      <c r="D5" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="L4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>46</v>
-      </c>
       <c r="E5" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G5" s="5"/>
       <c r="H5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="D6" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="J5" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="K5" s="4" t="s">
+      <c r="E6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="L5" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>60</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="5" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>68</v>
+        <v>195</v>
       </c>
       <c r="B8" s="3">
         <v>1674</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="3" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="K8" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="L8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>76</v>
-      </c>
       <c r="B9" s="5" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="5" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="I9" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="J9" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="L9" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M9" s="4" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="B10" s="3" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>94</v>
+        <v>74</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="G11" s="5"/>
       <c r="H11" s="5" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M11" s="4" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="G13" s="5"/>
       <c r="H13" s="5" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="L13" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M13" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="G15" s="5"/>
       <c r="H15" s="5" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="L15" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M15" s="4" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>135</v>
+        <v>118</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3" t="s">
-        <v>138</v>
+        <v>121</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>143</v>
+        <v>125</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>144</v>
+        <v>126</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>145</v>
+        <v>127</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="G17" s="5"/>
       <c r="H17" s="5" t="s">
-        <v>146</v>
+        <v>128</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>148</v>
+        <v>130</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M17" s="4" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>151</v>
+        <v>132</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>152</v>
+        <v>133</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3" t="s">
-        <v>154</v>
+        <v>135</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>155</v>
+        <v>136</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>155</v>
+        <v>136</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>156</v>
+        <v>137</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>159</v>
+        <v>139</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>161</v>
+        <v>141</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="G19" s="5"/>
       <c r="H19" s="5" t="s">
-        <v>162</v>
+        <v>142</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>163</v>
+        <v>143</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>163</v>
+        <v>143</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>164</v>
+        <v>144</v>
       </c>
       <c r="L19" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M19" s="4" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>166</v>
+        <v>152</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>167</v>
+        <v>146</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>168</v>
+        <v>147</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>169</v>
+        <v>148</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>170</v>
+        <v>149</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>171</v>
+        <v>150</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>171</v>
+        <v>150</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>172</v>
+        <v>151</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M20" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>175</v>
+        <v>153</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>176</v>
+        <v>154</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>177</v>
+        <v>155</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="5" t="s">
-        <v>178</v>
+        <v>156</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>179</v>
+        <v>157</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>179</v>
+        <v>157</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>180</v>
+        <v>158</v>
       </c>
       <c r="L21" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M21" s="4" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>183</v>
+        <v>160</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>184</v>
+        <v>161</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>185</v>
+        <v>162</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="3" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>188</v>
+        <v>165</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M22" s="2" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
-        <v>190</v>
+        <v>173</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>191</v>
+        <v>167</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>192</v>
+        <v>168</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>193</v>
+        <v>169</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G23" s="5"/>
       <c r="H23" s="5" t="s">
-        <v>194</v>
+        <v>170</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>195</v>
+        <v>171</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>195</v>
+        <v>171</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>196</v>
+        <v>172</v>
       </c>
       <c r="L23" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M23" s="4" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>199</v>
+        <v>174</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>201</v>
+        <v>176</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="3" t="s">
-        <v>202</v>
+        <v>177</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>203</v>
+        <v>178</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>203</v>
+        <v>178</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>204</v>
+        <v>179</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M24" s="2" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
-        <v>206</v>
+        <v>187</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>207</v>
+        <v>181</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>208</v>
+        <v>182</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>209</v>
+        <v>183</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G25" s="5"/>
       <c r="H25" s="5" t="s">
-        <v>210</v>
+        <v>184</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>211</v>
+        <v>185</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>211</v>
+        <v>185</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>212</v>
+        <v>186</v>
       </c>
       <c r="L25" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M25" s="4" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>214</v>
+        <v>194</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>215</v>
+        <v>188</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>216</v>
+        <v>189</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>217</v>
+        <v>190</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3" t="s">
-        <v>218</v>
+        <v>191</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>219</v>
+        <v>192</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>219</v>
+        <v>192</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>220</v>
+        <v>193</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>221</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix phase 7 rolls 1671/1674 and switch cohort photos to HQ PNGs.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/student/evening-students/7_phase/eveving cs enginering and medical_governmner.xlsx
+++ b/public/student/evening-students/7_phase/eveving cs enginering and medical_governmner.xlsx
@@ -933,10 +933,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>1670.png</v>
+        <v>1674.png</v>
       </c>
       <c r="B15" t="str">
-        <v>1670</v>
+        <v>1674</v>
       </c>
       <c r="C15" t="str">
         <v>M. Umar Ali</v>

</xml_diff>